<commit_message>
docs: six owner-defined roles; floor allocation stays pending (round 6)
- OD-32: floor allocation stays pending (exact floors not known);
  floors are entered later, consistent with OD-30.
- OD-33: roles are Super Admin, Operations Manager, Property Manager,
  Sales/CRM Executive, Marketing Manager and Finance, superseding the
  13 drafted roles. Permission matrix rebuilt with a mapping of the
  former roles; separation of duties is per person, with the Super
  Admin as second approver where only one person holds a role.
- Role terminology updated in the PRD, business rules, IA journeys,
  architecture, ERD (property_manager_id), pricing proposal and tests.
- Import template SG-INV-1.3: centre_manager_email renamed
  property_manager_email (no structural change; fixtures regenerated).
- Proposals Q-OW-13 (sales oversight duties) and Q-OW-14 (3D model
  upload) raised for confirmation.

Phase 1 remains IN PROGRESS.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/Fixtures/Inventory/SYNTHETIC_inventory_valid.xlsx
+++ b/tests/Fixtures/Inventory/SYNTHETIC_inventory_valid.xlsx
@@ -556,7 +556,7 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Template SG-INV-1.2 · draft generated 2026-10-24 · status: DRAFT; floors per property still to be supplied (Q-OW-1). Each address is its own property; current properties are owned and operated.</t>
+          <t>Template SG-INV-1.3 · draft generated 2026-10-24 · status: DRAFT; floors per property still to be supplied (Q-OW-1). Each address is its own property; current properties are owned and operated.</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>SG-INV-1.2</t>
+          <t>SG-INV-1.3</t>
         </is>
       </c>
     </row>
@@ -1230,7 +1230,7 @@
       </c>
       <c r="I1" s="7" t="inlineStr">
         <is>
-          <t>centre_manager_email</t>
+          <t>property_manager_email</t>
         </is>
       </c>
     </row>
@@ -1277,7 +1277,7 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Optional. Work email of the SmartGro centre manager (staff only).</t>
+          <t>Optional. Work email of the SmartGro Property Manager (staff only).</t>
         </is>
       </c>
     </row>

</xml_diff>